<commit_message>
rough initial work for first 3 metrics
</commit_message>
<xml_diff>
--- a/references/project timeline plan.xlsx
+++ b/references/project timeline plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\amelia\school\genAI\project\CS614-Generative-AI-with-LLMs\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C56256C-6D45-48FC-9881-E7E484161603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A9DDD2-5105-4AEC-B684-5569312D7B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4CC0CE9-BDAC-4C8D-8AD5-B79F55F8F7FA}"/>
   </bookViews>
@@ -81,16 +81,19 @@
 Reviewer: Amelia</t>
   </si>
   <si>
+    <t>Come up with agentic extension</t>
+  </si>
+  <si>
+    <t>Initial work: Amelia
+Refinement: Kavya
+generation : Akshit
+Reviewer: Kavya</t>
+  </si>
+  <si>
     <t>Initial work: Akshit
-Reviewer: Amelia</t>
-  </si>
-  <si>
-    <t>Initial work: Amelia
-Refinement + generation: Kavya
+Refinement: Amelia
+generation : Akshit
 Reviewer: Kavya</t>
-  </si>
-  <si>
-    <t>Come up with agentic extension</t>
   </si>
 </sst>
 </file>
@@ -213,6 +216,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -229,9 +235,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -569,14 +572,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025CEECF-55EA-4140-82C9-65F9BDCD0EDD}">
   <dimension ref="A2:U12"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38" style="3" customWidth="1"/>
     <col min="2" max="5" width="9.140625" style="3" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2">
         <v>46309</v>
@@ -639,15 +642,15 @@
         <v>46328</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="5"/>
@@ -666,16 +669,16 @@
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="14"/>
       <c r="F4" s="4"/>
       <c r="G4" s="5"/>
       <c r="H4" s="2"/>
@@ -693,22 +696,22 @@
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
+        <v>13</v>
+      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="12"/>
-      <c r="K5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="14"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -720,7 +723,7 @@
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
     </row>
-    <row r="6" spans="1:21" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -728,12 +731,12 @@
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="14"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -747,7 +750,7 @@
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
     </row>
-    <row r="7" spans="1:21" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -757,11 +760,11 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J7" s="9"/>
-      <c r="K7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="11"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
@@ -773,7 +776,7 @@
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
     </row>
-    <row r="8" spans="1:21" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -785,12 +788,12 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="11"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -800,7 +803,7 @@
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
     </row>
-    <row r="9" spans="1:21" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -812,12 +815,12 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="10"/>
+      <c r="J9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="11"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
@@ -827,7 +830,7 @@
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -843,10 +846,10 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="8" t="s">
+      <c r="N10" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="O10" s="10"/>
+      <c r="O10" s="11"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
@@ -854,7 +857,7 @@
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
     </row>
-    <row r="11" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
@@ -872,16 +875,16 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="8" t="s">
+      <c r="P11" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="11"/>
       <c r="U11" s="1"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -910,15 +913,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="I5:K5"/>
     <mergeCell ref="J9:M9"/>
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="P11:T11"/>
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="F6:I6"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="I5:K5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
script to call elephant metrics
</commit_message>
<xml_diff>
--- a/references/project timeline plan.xlsx
+++ b/references/project timeline plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\amelia\school\genAI\project\CS614-Generative-AI-with-LLMs\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A9DDD2-5105-4AEC-B684-5569312D7B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F56DF9-2CC6-456B-8D77-EA1A150E3016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4CC0CE9-BDAC-4C8D-8AD5-B79F55F8F7FA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Dataset generation</t>
   </si>
@@ -71,29 +71,36 @@
     <t>All - independently</t>
   </si>
   <si>
+    <t>Come up with agentic extension</t>
+  </si>
+  <si>
+    <t>Amelia</t>
+  </si>
+  <si>
+    <t>Initial work: Amelia
+Refinement + generation: Akshit</t>
+  </si>
+  <si>
+    <t>Intial work: Amelia
+Refinement + generation: Akshit</t>
+  </si>
+  <si>
     <t>proprietary models: Akshit 
-open-source models: Kavya
-Reviewer: Amelia</t>
-  </si>
-  <si>
-    <t>Intial work: Amelia
-Refinement + generation: Akshit
-Reviewer: Amelia</t>
-  </si>
-  <si>
-    <t>Come up with agentic extension</t>
-  </si>
-  <si>
-    <t>Initial work: Amelia
-Refinement: Kavya
-generation : Akshit
-Reviewer: Kavya</t>
-  </si>
-  <si>
-    <t>Initial work: Akshit
-Refinement: Amelia
-generation : Akshit
-Reviewer: Kavya</t>
+open-source models: Kavya</t>
+  </si>
+  <si>
+    <t>Initial work: Kavya
+Refinement + generation: Akshit</t>
+  </si>
+  <si>
+    <t>Answering agent</t>
+  </si>
+  <si>
+    <t>Akshit
+Kavya</t>
+  </si>
+  <si>
+    <t>Comile results</t>
   </si>
 </sst>
 </file>
@@ -129,7 +136,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -189,11 +196,46 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -219,6 +261,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -228,13 +279,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025CEECF-55EA-4140-82C9-65F9BDCD0EDD}">
-  <dimension ref="A2:U12"/>
+  <dimension ref="A2:U14"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" style="3" customWidth="1"/>
@@ -646,11 +700,11 @@
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="14"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="5"/>
@@ -673,12 +727,12 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="14"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="5"/>
       <c r="H4" s="2"/>
@@ -698,7 +752,7 @@
     </row>
     <row r="5" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -707,11 +761,11 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="13"/>
-      <c r="K5" s="14"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="11"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -723,7 +777,7 @@
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
     </row>
-    <row r="6" spans="1:21" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -731,12 +785,12 @@
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
-      <c r="F6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="14"/>
+      <c r="F6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -750,7 +804,7 @@
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
     </row>
-    <row r="7" spans="1:21" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -760,15 +814,15 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="I7" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="10"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
+      <c r="I7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="14"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
@@ -776,7 +830,7 @@
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
     </row>
-    <row r="8" spans="1:21" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -788,22 +842,22 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
     </row>
-    <row r="9" spans="1:21" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -815,15 +869,15 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="14"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -831,35 +885,35 @@
       <c r="U9" s="1"/>
     </row>
     <row r="10" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="O10" s="11"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="1"/>
-      <c r="U10" s="1"/>
-    </row>
-    <row r="11" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+    </row>
+    <row r="11" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -875,18 +929,18 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="10"/>
-      <c r="S11" s="10"/>
-      <c r="T11" s="11"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="R11" s="14"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
       <c r="U11" s="1"/>
     </row>
-    <row r="12" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -905,23 +959,79 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="1"/>
-      <c r="U12" s="7" t="s">
+      <c r="S12" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="T12" s="18"/>
+      <c r="U12" s="1"/>
+    </row>
+    <row r="13" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="12" t="s">
         <v>7</v>
       </c>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="13"/>
+      <c r="S13" s="13"/>
+      <c r="T13" s="14"/>
+      <c r="U13" s="1"/>
+    </row>
+    <row r="14" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="P13:T13"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="I7:O7"/>
+    <mergeCell ref="L8:P8"/>
+    <mergeCell ref="L9:P9"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="S12:T12"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="J8:M8"/>
     <mergeCell ref="I5:K5"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="P11:T11"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="F6:I6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
compilation of results with original prompt
</commit_message>
<xml_diff>
--- a/references/project timeline plan.xlsx
+++ b/references/project timeline plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\amelia\school\genAI\project\CS614-Generative-AI-with-LLMs\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1CAC28-9EAD-459E-BEC5-11631DA0B9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F03D1E-F42B-424D-95DA-F5BC15E03A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4CC0CE9-BDAC-4C8D-8AD5-B79F55F8F7FA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Dataset generation</t>
   </si>
@@ -50,13 +50,7 @@
     <t>Run the BASIL metrics</t>
   </si>
   <si>
-    <t>Compile the results</t>
-  </si>
-  <si>
     <t>Prepare for the presentation and report</t>
-  </si>
-  <si>
-    <t>Presentation and report due</t>
   </si>
   <si>
     <t>Read papers</t>
@@ -89,15 +83,21 @@
     <t>Answering agent</t>
   </si>
   <si>
-    <t>Akshit
-Kavya</t>
-  </si>
-  <si>
-    <t>Comile results</t>
-  </si>
-  <si>
     <t>Initial work + generation: Akshit
 Refinement: Amelia</t>
+  </si>
+  <si>
+    <t>Initial work: Kavya
+Refinement + generation: Akshit</t>
+  </si>
+  <si>
+    <t>Compile the results (elephant + basil)</t>
+  </si>
+  <si>
+    <t>Compile results (agent)</t>
+  </si>
+  <si>
+    <t>All</t>
   </si>
 </sst>
 </file>
@@ -133,7 +133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -206,33 +206,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -258,10 +236,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -271,15 +252,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -616,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025CEECF-55EA-4140-82C9-65F9BDCD0EDD}">
-  <dimension ref="A2:U14"/>
+  <dimension ref="A2:V13"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" style="3" customWidth="1"/>
@@ -624,7 +596,7 @@
     <col min="6" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2">
         <v>46309</v>
@@ -686,16 +658,19 @@
       <c r="U2" s="2">
         <v>46328</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V2" s="2">
+        <v>46329</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
+        <v>6</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="5"/>
@@ -713,17 +688,18 @@
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
-    </row>
-    <row r="4" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="16"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="4"/>
       <c r="G4" s="5"/>
       <c r="H4" s="2"/>
@@ -740,10 +716,11 @@
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V4" s="2"/>
+    </row>
+    <row r="5" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -752,11 +729,11 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="16"/>
+      <c r="I5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="10"/>
+      <c r="K5" s="11"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -767,8 +744,9 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V5" s="2"/>
+    </row>
+    <row r="6" spans="1:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -776,12 +754,12 @@
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
-      <c r="F6" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
+      <c r="F6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -794,8 +772,9 @@
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
-    </row>
-    <row r="7" spans="1:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V6" s="1"/>
+    </row>
+    <row r="7" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -805,23 +784,24 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="I7" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
-      <c r="O7" s="13"/>
+      <c r="I7" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="14"/>
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
-    </row>
-    <row r="8" spans="1:21" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V7" s="1"/>
+    </row>
+    <row r="8" spans="1:22" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -835,20 +815,21 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
-      <c r="L8" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
+      <c r="L8" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
       <c r="Q8" s="13"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
+      <c r="R8" s="13"/>
+      <c r="S8" s="14"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
-    </row>
-    <row r="9" spans="1:21" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -862,22 +843,23 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
-      <c r="L9" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
+      <c r="L9" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
       <c r="Q9" s="13"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
+      <c r="R9" s="13"/>
+      <c r="S9" s="14"/>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
-    </row>
-    <row r="10" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V9" s="1"/>
+    </row>
+    <row r="10" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -893,17 +875,19 @@
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="Q10" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="R10" s="13"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="T10" s="14"/>
       <c r="U10" s="8"/>
-    </row>
-    <row r="11" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V10" s="8"/>
+    </row>
+    <row r="11" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -920,15 +904,16 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
-      <c r="Q11" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="R11" s="12"/>
+      <c r="Q11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="R11" s="13"/>
       <c r="S11" s="13"/>
-      <c r="T11" s="1"/>
+      <c r="T11" s="14"/>
       <c r="U11" s="1"/>
-    </row>
-    <row r="12" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V11" s="1"/>
+    </row>
+    <row r="12" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -949,15 +934,14 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
-      <c r="S12" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="T12" s="10"/>
+      <c r="S12" s="1"/>
+      <c r="T12" s="1"/>
       <c r="U12" s="1"/>
-    </row>
-    <row r="13" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="V12" s="1"/>
+    </row>
+    <row r="13" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -976,47 +960,25 @@
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
-    </row>
-    <row r="14" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="1"/>
-      <c r="U14" s="1"/>
+      <c r="S13" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="T13" s="13"/>
+      <c r="U13" s="13"/>
+      <c r="V13" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="S13:V13"/>
+    <mergeCell ref="S10:T10"/>
+    <mergeCell ref="L8:S8"/>
+    <mergeCell ref="L9:S9"/>
+    <mergeCell ref="Q11:T11"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="I5:K5"/>
-    <mergeCell ref="L8:Q8"/>
-    <mergeCell ref="L9:Q9"/>
     <mergeCell ref="F6:I6"/>
     <mergeCell ref="I7:O7"/>
-    <mergeCell ref="S12:T12"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q11:S11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>